<commit_message>
Support multiple family groups per device, admin member/group removal, and outside-tap dialog close
- Change group membership from one-per-device to one-per-device-per-group, so a device can join multiple groups and no longer gets silently duplicated when local storage is lost
- Let admins remove other members and delete a whole group (native + web)
- Replace the native admin status-change Alert with a custom bottom-sheet Modal that closes on outside tap, matching the web version
- Add a group switcher and "join another group" flow to Settings (native + web)
- Back up the web version's participation data to a cookie so it survives localStorage being cleared on iPhone
- Update design docs and test spec spreadsheets to match

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/設計書/テスト仕様書_API.xlsx
+++ b/設計書/テスト仕様書_API.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1332,6 +1332,222 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>/groups/join</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>複数グループへの参加(別グループ)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>{"device_id":"dev-001","invite_code":"654321","name":"さくら"}</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>200 OK、group_id・member_idが返る(dev-001は既に別グループに参加済みだが、別グループへの参加は許可される)</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>F2/F18</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>/groups/join</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>同一グループへの重複参加</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>{"device_id":"dev-002","invite_code":"123456","name":"お母さん"}</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>409 ALREADY_JOINED、既に参加しているグループへの重複参加は拒否される</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>/members/:memberId</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>管理者による他メンバーの削除</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>対象メンバーとは別のdevice_id(管理者)をヘッダーに指定</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>200 OK、{ok:true}が返り、対象メンバーが一覧から削除される</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>/members/:memberId</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>管理者以外による他メンバー削除の拒否</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>対象メンバーとは別のdevice_id(管理者でない)をヘッダーに指定</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>403 FORBIDDEN、削除されない</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>/groups/:groupId</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>管理者によるグループ削除</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>ヘッダーに管理者のdevice_id</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>200 OK、{ok:true}が返り、グループと所属メンバー全員が削除される</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>F20</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>/groups/:groupId</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>管理者以外によるグループ削除の拒否</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>ヘッダーに管理者でないdevice_id</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>403 FORBIDDEN、グループは削除されない</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>F20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sync participating groups from the DB instead of trusting device storage alone
- Add GET /memberships so a device can ask the server which groups it actually belongs to
- Refresh the local group list from this endpoint on app boot and whenever Settings is opened (native), and on load/refresh (web), so a device recovers its memberships even after storage is lost or a reinstall
- Show each group's invite code in the switcher list so groups with the same display name are easy to tell apart
- Update design docs and test specs to match

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/設計書/テスト仕様書_API.xlsx
+++ b/設計書/テスト仕様書_API.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1548,6 +1548,78 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>/memberships</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>参加中グループ一覧のDB取得</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>ヘッダーにdevice_id</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>200 OK、その端末が参加している全グループの{groupId,memberId,myName,inviteCode}配列が返る</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>F18</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>/memberships</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>参加しているグループが無い端末での取得</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>ヘッダーに未登録のdevice_id</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>200 OK、空配列が返る</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>F18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add privacy policy and version display; fix a label overflow; let re-joining by name resume the same member
- Fix the building-radius label on the home registration screen getting clipped by giving it flex and letting it wrap instead of pushing the meter value off-screen
- Add a privacy policy (native screen + /privacy.html for the web fallback) and show the app version in Settings on both platforms
- When joining a group, if the name exactly matches an existing member in that group, re-link that member's device_id instead of creating a duplicate — lets someone recover their identity (status, admin flag, home location) after reinstalling instead of ending up as an orphaned duplicate entry
- Update design docs and test specs to match

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/設計書/テスト仕様書_API.xlsx
+++ b/設計書/テスト仕様書_API.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1656,6 +1656,42 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>/groups/join</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>同じ名前での再参加(端末の再インストール等からの復帰)</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>{"device_id":"新しいdevice_id","inviteCode":"既存グループのコード","name":"以前と同じ名前"}</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>200 OK、同じmember_idが返る。device_idのみ更新され、状態や管理者権限は引き継がれる。重複登録はされない</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Suppress notification and arrival/departure time when an admin forces a status change
A member's status display now hides the "18:32に帰宅"-style time and skips
pushing a notification when the change came from an admin acting on their
behalf, since it isn't the member's own real arrival/departure. Self-made
changes keep working exactly as before.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/設計書/テスト仕様書_API.xlsx
+++ b/設計書/テスト仕様書_API.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1692,6 +1692,114 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>/members/:memberId/status</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>管理者が代理変更した場合、本人以外への通知が送られない</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>{"device_id":"管理者のdevice_id","status":"home"}(対象memberIdは別メンバー)</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>200 OK。対象メンバーのstatusは更新されるが、通知設定ONの他メンバーにもプッシュ通知は送信されない</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>F12</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>/members/:memberId/status</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>管理者が代理変更した場合、status_updated_atが更新されない</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>{"device_id":"管理者のdevice_id","status":"home"}(対象memberIdは別メンバー)</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>200 OK。対象メンバーのstatus_updated_atは変更前の値のまま。一覧取得時のstatusSetByAdminがtrueになる</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>F12</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>/members/:memberId/status</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>本人が自分で変更した場合は、従来どおり通知が送られ、statusSetByAdminはfalseのままになる</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>{"device_id":"本人のdevice_id","status":"home"}</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>200 OK。通知設定ONの他メンバーに通知が送られ、一覧取得時のstatusSetByAdminはfalse</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>F12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>